<commit_message>
feat(F-NAR-019): TREE-DIF-033 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-033.xlsx
+++ b/stories/arbres/TREE-DIF-033.xlsx
@@ -3095,17 +3095,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, le ticket sur le genou. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. Le ticket bleu ne bouge plus. Maintenant, c'est à nous.</t>
+          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, le ticket sur le genou. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. Le ticket bleu ne bouge plus. Maintenant, c'est à nous.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt; sur le genou. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. Le ticket bleu ne bouge plus. Maintenant, c'est à nous.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt; sur le genou. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. Le ticket bleu ne bouge plus. Maintenant, c'est à nous.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, le &lt;emphasis&gt;ticket&lt;/emphasis&gt; sur le genou. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. Le ticket bleu ne bouge plus. Maintenant, c'est à nous. [pause]</t>
+          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, le &lt;emphasis&gt;ticket&lt;/emphasis&gt; sur le genou. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. Le ticket bleu ne bouge plus. Maintenant, c'est à nous. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3242,7 +3242,7 @@
           <t>enfant-f|On attend un peu, Aniss.
 enfant-m|J'attends, je souffle.
 narrateur|Aniss s'assoit près du kiosque, le ticket sur le genou.
-narrateur|La file repose, toute ronde, toute sage.
+narrateur|La file repose, ronde comme le kiosque.
 narrateur|Sarah replace le pas, sans tirer.
 papa|Tes pieds ont su s'asseoir.
 maman|Le tour a eu la place.
@@ -3279,17 +3279,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. Le ticket bleu reste dans la paume de Sarah. Je reste un peu. Un pois de sucre colle aux cheveux d'Aniss.</t>
+          <t>Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. Le ticket bleu reste dans la paume de Sarah. Je reste un peu. Un pois de sucre colle aux cheveux d'Aniss.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. Le ticket bleu reste dans la paume de Sarah. Je reste un peu. Un pois de sucre colle aux cheveux d'Aniss.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. Le ticket bleu reste dans la paume de Sarah. Je reste un peu. Un pois de sucre colle aux cheveux d'Aniss.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. Le ticket bleu reste dans la paume de Sarah. Je reste un peu. Un pois de sucre colle aux cheveux d'Aniss.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. Le ticket bleu reste dans la paume de Sarah. Je reste un peu. Un pois de sucre colle aux cheveux d'Aniss.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3427,9 +3427,9 @@
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>narrateur|Au bord de la file, deux têtes se calment.
+          <t>narrateur|Au bord de la file, deux têtes se posent.
 enfant-f|Aniss, tu as su t'asseoir.
-enfant-m|Oui, tout près de tes mains.
+enfant-m|Oui, contre tes mains.
 papa|Toi debout, lui assis, ça tenait.
 maman|Vos voix sont devenues toutes petites.
 narrateur|Le ticket bleu reste dans la paume de Sarah.
@@ -3466,17 +3466,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, hors de la file. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. Le ticket bleu reste près d'eux. La file est prête.</t>
+          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, hors de la file. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. Le ticket bleu reste près d'eux. La file est prête.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;, hors de la file. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. Le ticket bleu reste près d'eux. La file est prête.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;, hors de la file. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. Le ticket bleu reste près d'eux. La file est prête.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le &lt;emphasis&gt;ticket&lt;/emphasis&gt;, hors de la file. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. Le ticket bleu reste près d'eux. La file est prête. [pause]</t>
+          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le &lt;emphasis&gt;ticket&lt;/emphasis&gt;, hors de la file. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. Le ticket bleu reste près d'eux. La file est prête. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3616,7 +3616,7 @@
 narrateur|Les mains d'Aniss sont libres, maintenant.
 narrateur|Sarah avance d'un pas, pile au milieu.
 enfant-m|Je t'aide, sans le ticket.
-maman|Vous avez demandé, et ça tient.
+maman|Papa a le papier, vos mains sont libres.
 narrateur|Le ticket bleu reste près d'eux.
 enfant-f|La file est prête.</t>
         </is>
@@ -3837,17 +3837,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le ticket près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. Le ticket frôle le bois, trop bas. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Sarah pose le ticket près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. Le ticket frôle le bois, trop bas. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose le ticket près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. Le ticket frôle le bois, trop bas. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose le ticket près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. Le ticket frôle le bois, trop bas. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah pose le ticket près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. Le ticket frôle le bois, trop bas. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah pose le ticket près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. Le ticket frôle le bois, trop bas. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3993,7 +3993,7 @@
 narrateur|Le ticket frôle le bois, trop bas.
 narrateur|Un peu de poussière lève, puis retombe.
 narrateur|Sarah se cogne à son épaule, surprise.
-maman|Il a de l'élan, comme un petit vent.
+maman|Ses pieds veulent le haut, avant toi.
 papa|Toi tu as les jambes plus longues.
 enfant-f|On peut jouer avec lui ?
 papa|Vous trouvez, tous les deux ?</t>
@@ -4224,17 +4224,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose le ticket, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer.</t>
+          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose le ticket, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose le &lt;emphasis&gt;ticket&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer. [pause]</t>
+          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose le &lt;emphasis&gt;ticket&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4375,7 +4375,7 @@
 narrateur|Aniss va plus vite, Sarah plus loin.
 enfant-f|On arrive en haut, tous les deux.
 enfant-m|J'ai attendu ta jambe, un peu.
-papa|Vous avez joué avec l'élan.
+papa|Vos ombres ont monté ensemble.
 maman|Le marchepied vous a laissés passer.</t>
         </is>
       </c>
@@ -4596,17 +4596,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient le ticket, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois.</t>
+          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient le ticket, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient le &lt;emphasis&gt;ticket&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois. [pause]</t>
+          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient le &lt;emphasis&gt;ticket&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4748,7 +4748,7 @@
 enfant-m|C'est à toi, Sarah.
 enfant-f|Merci, j'y vais.
 papa|Chacun son tour, sur la marche.
-maman|L'élan a attendu le bois.</t>
+maman|Ses genoux ont reposé sur le bois.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -4967,17 +4967,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près du ticket. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu.</t>
+          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près du ticket. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près du &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près du &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près du &lt;emphasis&gt;ticket&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu. [pause]</t>
+          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près du &lt;emphasis&gt;ticket&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5118,7 +5118,7 @@
 narrateur|Sarah la reçoit, monte plus loin.
 enfant-m|On demande, et ça va !
 enfant-f|Le haut est à nous.
-papa|Vous avez demandé, sans tirer.
+papa|Ma main tenait, vous montiez.
 maman|Ma main a juste attendu.</t>
         </is>
       </c>
@@ -5151,17 +5151,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. Le ticket bleu marque le bois, une petite ligne. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le pois reste au chaud, sur la marche.</t>
+          <t>Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. Le ticket bleu marque le bois, une petite ligne. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le pois reste au chaud, sur la marche.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. Le ticket bleu marque le bois, une petite ligne. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le pois reste au chaud, sur la marche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. Le ticket bleu marque le bois, une petite ligne. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le pois reste au chaud, sur la marche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. Le ticket bleu marque le bois, une petite ligne. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le pois reste au chaud, sur la marche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. Le ticket bleu marque le bois, une petite ligne. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le pois reste au chaud, sur la marche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5303,7 +5303,7 @@
 enfant-f|Maman a tendu l'écharpe.
 enfant-m|On s'est parlé à travers.
 papa|Le marchepied vous a laissé la place.
-maman|Le secret tient, tout chaud.
+maman|Le secret tient, chaud dans les mains.
 narrateur|Le ticket bleu marque le bois, une petite ligne.
 enfant-f|Regarde-le, Aniss, il brille.
 enfant-m|Je le vois, d'ici.
@@ -5339,17 +5339,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Sarah glisse le ticket près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. Le ticket frôle l'or, trop vite. Le ticket attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Sarah glisse le ticket près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. Le ticket frôle l'or, trop vite. Le ticket attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah glisse le ticket près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. Le ticket frôle l'or, trop vite. Le ticket attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah glisse le ticket près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. Le ticket frôle l'or, trop vite. Le ticket attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah glisse le ticket près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. Le ticket frôle l'or, trop vite. Le ticket attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah glisse le ticket près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. Le ticket frôle l'or, trop vite. Le ticket attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5491,11 +5491,11 @@
 enfant-f|Ici, ça brille, Aniss.
 enfant-f|Tu t'assois, et on tourne.
 enfant-m|Je galope, trop fort !
-narrateur|Le cheval doré penche, un tout petit peu.
+narrateur|Le cheval doré penche, un petit peu.
 narrateur|Le ticket frôle l'or, trop vite.
 narrateur|Le ticket attend au bord, un peu seule.
 narrateur|Sarah serre la selle, les dents serrées.
-maman|Son élan remplit tout le tour.
+maman|Ses genoux tapent la selle, trop fort.
 papa|Toi tu vas plus loin, lui plus vite.
 enfant-m|On tourne comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
@@ -5910,17 +5910,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La crinière sent le vernis, tout près. Le tour est à vous, maintenant. Le ticket bleu pèse dans la poche, un peu lourd. Sarah la pose contre le bois peint. Un rai d'or traverse le ticket, dans la poche.</t>
+          <t>Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La crinière sent le vernis, sous le nez. Le tour est à vous, maintenant. Le ticket bleu pèse dans la poche, un peu lourd. Sarah la pose contre le bois peint. Un rai d'or traverse le ticket, dans la poche.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis level="moderate"&gt;crinière&lt;/emphasis&gt; sent le vernis, tout près. Le tour est à vous, maintenant. Le ticket bleu pèse dans la poche, un peu lourd. Sarah la pose contre le bois peint. Un rai d'or traverse le ticket, dans la poche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis level="moderate"&gt;crinière&lt;/emphasis&gt; sent le vernis, sous le nez. Le tour est à vous, maintenant. Le ticket bleu pèse dans la poche, un peu lourd. Sarah la pose contre le bois peint. Un rai d'or traverse le ticket, dans la poche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis&gt;crinière&lt;/emphasis&gt; sent le vernis, tout près. Le tour est à vous, maintenant. Le ticket bleu pèse dans la poche, un peu lourd. Sarah la pose contre le bois peint. Un rai d'or traverse le ticket, dans la poche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis&gt;crinière&lt;/emphasis&gt; sent le vernis, sous le nez. Le tour est à vous, maintenant. Le ticket bleu pèse dans la poche, un peu lourd. Sarah la pose contre le bois peint. Un rai d'or traverse le ticket, dans la poche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6061,7 +6061,7 @@
           <t>narrateur|Les talons d'Aniss sont chauds, sur le bois.
 enfant-f|Tu as chanté pour moi.
 enfant-m|Tu tenais mon épaule.
-maman|La crinière sent le vernis, tout près.
+maman|La crinière sent le vernis, sous le nez.
 papa|Le tour est à vous, maintenant.
 narrateur|Le ticket bleu pèse dans la poche, un peu lourd.
 narrateur|Sarah la pose contre le bois peint.
@@ -6097,17 +6097,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. Le ticket bleu reste muet, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois.</t>
+          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. Le ticket bleu reste muet, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'arrêt. Quand il s'arrête, on galope un peu. Le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt; bleu reste muet, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'arrêt. Quand il s'arrête, on galope un peu. Le &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt; bleu reste muet, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. Le &lt;emphasis&gt;ticket&lt;/emphasis&gt; bleu reste muet, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois. [pause]</t>
+          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. Le &lt;emphasis&gt;ticket&lt;/emphasis&gt; bleu reste muet, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6244,12 +6244,12 @@
           <t>enfant-f|On attend l'arrêt.
 enfant-m|Quand il s'arrête, on galope un peu.
 narrateur|Le ticket bleu reste muet, au creux.
-narrateur|Le cheval doré ralentit, tout seul.
+narrateur|Le cheval doré ralentit, sans nous.
 narrateur|Aniss souffle, puis il ouvre les mains.
 enfant-m|C'est à nous, maintenant.
 enfant-f|Un tour, sans galoper.
 papa|Vous avez attendu la musique.
-maman|L'élan a écouté le bois.</t>
+maman|Ses mains ont attendu le bois.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
@@ -6469,17 +6469,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près du ticket. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu.</t>
+          <t>Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près du ticket. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près du &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près du &lt;emphasis level="moderate"&gt;ticket&lt;/emphasis&gt;. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près du &lt;emphasis&gt;ticket&lt;/emphasis&gt;. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu. [pause]</t>
+          <t>Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près du &lt;emphasis&gt;ticket&lt;/emphasis&gt;. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6614,13 +6614,13 @@
       <c r="AW30" t="inlineStr">
         <is>
           <t>enfant-f|Papa, tu tiens la barre ?
-papa|Je la tiens, tout ferme.
+papa|Je la tiens, bien ferme.
 narrateur|Papa tient la barre, près du ticket.
-narrateur|Aniss pose les deux mains, tout près.
+narrateur|Aniss pose les deux mains, contre la barre.
 narrateur|Sarah pose les siennes, plus loin.
 enfant-m|On demande, et ça tient !
 enfant-f|La crinière est à nous.
-maman|Vous avez demandé, sans galoper.
+maman|La barre tient, le cheval aussi.
 papa|Ma barre a juste attendu.</t>
         </is>
       </c>
@@ -6841,17 +6841,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Sarah enroule l'écharpe à pois autour du cou. Pour le vent du tour, Aniss ! Je tourne, moi aussi ! Aniss tourne trop vite, et un pois s'accroche. L'écharpe tire, Sarah recule d'un pas. Aïe, attends ! Autour du cou, sans danser. Sarah noue le tissu, un pois contre le pull. Le ticket et la clochette voyagent avec vous. Aniss prend la clochette, genoux plus vifs. On y va, mais le pois reste.</t>
+          <t>Sarah enroule l'écharpe à pois autour du cou. Pour le vent du tour, Aniss ! Je tourne, moi aussi ! Aniss tourne trop vite, et un pois s'accroche. L'écharpe tire, Sarah recule d'un pas. Aïe, attends ! Autour du cou, le pois contre le pull. Sarah noue le tissu, un pois contre le pull. Le ticket et la clochette voyagent avec vous. Aniss prend la clochette, genoux plus vifs. On y va, mais le pois reste.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah enroule l'&lt;emphasis level="moderate"&gt;écharpe à pois&lt;/emphasis&gt; autour du cou. Pour le vent du tour, Aniss ! Je tourne, moi aussi ! Aniss tourne trop vite, et un pois s'accroche. L'écharpe tire, Sarah recule d'un pas. Aïe, attends ! Autour du cou, sans danser. Sarah noue le tissu, un pois contre le pull. Le ticket et la clochette voyagent avec vous. Aniss prend la clochette, genoux plus vifs. On y va, mais le pois reste.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah enroule l'&lt;emphasis level="moderate"&gt;écharpe à pois&lt;/emphasis&gt; autour du cou. Pour le vent du tour, Aniss ! Je tourne, moi aussi ! Aniss tourne trop vite, et un pois s'accroche. L'écharpe tire, Sarah recule d'un pas. Aïe, attends ! Autour du cou, le pois contre le pull. Sarah noue le tissu, un pois contre le pull. Le ticket et la clochette voyagent avec vous. Aniss prend la clochette, genoux plus vifs. On y va, mais le pois reste.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Sarah enroule l'&lt;emphasis&gt;écharpe à pois&lt;/emphasis&gt; autour du cou. Pour le vent du tour, Aniss ! Je tourne, moi aussi ! Aniss tourne trop vite, et un pois s'accroche. L'écharpe tire, Sarah recule d'un pas. Aïe, attends ! Autour du cou, sans danser. Sarah noue le tissu, un pois contre le pull. Le ticket et la clochette voyagent avec vous. Aniss prend la clochette, genoux plus vifs. On y va, mais le pois reste. [pause]</t>
+          <t>Sarah enroule l'&lt;emphasis&gt;écharpe à pois&lt;/emphasis&gt; autour du cou. Pour le vent du tour, Aniss ! Je tourne, moi aussi ! Aniss tourne trop vite, et un pois s'accroche. L'écharpe tire, Sarah recule d'un pas. Aïe, attends ! Autour du cou, le pois contre le pull. Sarah noue le tissu, un pois contre le pull. Le ticket et la clochette voyagent avec vous. Aniss prend la clochette, genoux plus vifs. On y va, mais le pois reste. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6991,7 +6991,7 @@
 narrateur|Aniss tourne trop vite, et un pois s'accroche.
 narrateur|L'écharpe tire, Sarah recule d'un pas.
 enfant-f|Aïe, attends !
-papa|Autour du cou, sans danser.
+papa|Autour du cou, le pois contre le pull.
 narrateur|Sarah noue le tissu, un pois contre le pull.
 maman|Le ticket et la clochette voyagent avec vous.
 narrateur|Aniss prend la clochette, genoux plus vifs.
@@ -7215,17 +7215,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Le cou porte l'écharpe, contre le pull. Elle a trop de pois ! C'est pour le vent du tour. Les pieds d'Aniss tapent le sol peint. Merci, tu as noué le pois sans danser. On reste près des chevaux ? Oui, papa.</t>
+          <t>Le cou porte l'écharpe, contre le pull. Elle a trop de pois ! C'est pour le vent du tour. Les pieds d'Aniss tapent le sol peint. Merci, le pois tient contre le pull. On reste près des chevaux ? Oui, papa.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cou porte l'écharpe, contre le pull. Elle a trop de pois ! C'est pour le vent du tour. Les pieds d'Aniss tapent le sol peint. &lt;emphasis level="moderate"&gt;Merci&lt;/emphasis&gt;, tu as noué le pois sans danser. On reste près des chevaux ? Oui, papa.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cou porte l'écharpe, contre le pull. Elle a trop de pois ! C'est pour le vent du tour. Les pieds d'Aniss tapent le sol peint. &lt;emphasis level="moderate"&gt;Merci&lt;/emphasis&gt;, le pois tient contre le pull. On reste près des chevaux ? Oui, papa.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Le cou porte l'écharpe, contre le pull. Elle a trop de pois ! C'est pour le vent du tour. Les pieds d'Aniss tapent le sol peint. &lt;emphasis&gt;Merci&lt;/emphasis&gt;, tu as noué le pois sans danser. On reste près des chevaux ? Oui, papa. [pause]</t>
+          <t>Le cou porte l'écharpe, contre le pull. Elle a trop de pois ! C'est pour le vent du tour. Les pieds d'Aniss tapent le sol peint. &lt;emphasis&gt;Merci&lt;/emphasis&gt;, le pois tient contre le pull. On reste près des chevaux ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7363,7 +7363,7 @@
 enfant-m|Elle a trop de pois !
 enfant-f|C'est pour le vent du tour.
 narrateur|Les pieds d'Aniss tapent le sol peint.
-maman|Merci, tu as noué le pois sans danser.
+maman|Merci, le pois tient contre le pull.
 papa|On reste près des chevaux ?
 enfant-f|Oui, papa.</t>
         </is>
@@ -8349,17 +8349,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, un pois sous la main. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. L'écharpe à pois ne bouge plus. Maintenant, c'est à nous.</t>
+          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, un pois sous la main. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. L'écharpe à pois ne bouge plus. Maintenant, c'est à nous.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, un pois sous la main. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. L'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt; à pois ne bouge plus. Maintenant, c'est à nous.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, un pois sous la main. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. L'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt; à pois ne bouge plus. Maintenant, c'est à nous.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, un pois sous la main. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. L'&lt;emphasis&gt;écharpe&lt;/emphasis&gt; à pois ne bouge plus. Maintenant, c'est à nous. [pause]</t>
+          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, un pois sous la main. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. L'&lt;emphasis&gt;écharpe&lt;/emphasis&gt; à pois ne bouge plus. Maintenant, c'est à nous. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8496,7 +8496,7 @@
           <t>enfant-f|On attend un peu, Aniss.
 enfant-m|J'attends, je souffle.
 narrateur|Aniss s'assoit près du kiosque, un pois sous la main.
-narrateur|La file repose, toute ronde, toute sage.
+narrateur|La file repose, ronde comme le kiosque.
 narrateur|Sarah replace le pas, sans tirer.
 papa|Tes pieds ont su s'asseoir.
 maman|Le tour a eu la place.
@@ -8533,17 +8533,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. L'écharpe à pois reste dans la paume de Sarah. Je reste un peu. Le kiosque sent la gaufre, et le pois se tait.</t>
+          <t>Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. L'écharpe à pois reste dans la paume de Sarah. Je reste un peu. Le kiosque sent la gaufre, et le pois se tait.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. L'écharpe à pois reste dans la paume de Sarah. Je reste un peu. Le kiosque sent la gaufre, et le pois se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. L'écharpe à pois reste dans la paume de Sarah. Je reste un peu. Le kiosque sent la gaufre, et le pois se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. L'écharpe à pois reste dans la paume de Sarah. Je reste un peu. Le kiosque sent la gaufre, et le pois se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. L'écharpe à pois reste dans la paume de Sarah. Je reste un peu. Le kiosque sent la gaufre, et le pois se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8681,9 +8681,9 @@
       </c>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Au bord de la file, deux têtes se calment.
+          <t>narrateur|Au bord de la file, deux têtes se posent.
 enfant-f|Aniss, tu as su t'asseoir.
-enfant-m|Oui, tout près de tes mains.
+enfant-m|Oui, contre tes mains.
 papa|Toi debout, lui assis, ça tenait.
 maman|Vos voix sont devenues toutes petites.
 narrateur|L'écharpe à pois reste dans la paume de Sarah.
@@ -8720,17 +8720,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, près de l'écharpe. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. L'écharpe à pois reste près d'eux. La file est prête.</t>
+          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, près de l'écharpe. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. L'écharpe à pois reste près d'eux. La file est prête.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, près de l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. L'écharpe à pois reste près d'eux. La file est prête.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, près de l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. L'écharpe à pois reste près d'eux. La file est prête.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, près de l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. L'écharpe à pois reste près d'eux. La file est prête. [pause]</t>
+          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, près de l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. L'écharpe à pois reste près d'eux. La file est prête. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8870,7 +8870,7 @@
 narrateur|Les mains d'Aniss sont libres, maintenant.
 narrateur|Sarah avance d'un pas, pile au milieu.
 enfant-m|Je t'aide, sans le ticket.
-maman|Vous avez demandé, et ça tient.
+maman|Papa a le papier, vos mains sont libres.
 narrateur|L'écharpe à pois reste près d'eux.
 enfant-f|La file est prête.</t>
         </is>
@@ -9091,17 +9091,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose l'écharpe près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. L'écharpe accroche une vis, un instant. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Sarah pose l'écharpe près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. L'écharpe accroche une vis, un instant. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose l'écharpe près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. L'écharpe accroche une vis, un instant. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose l'écharpe près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. L'écharpe accroche une vis, un instant. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah pose l'écharpe près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. L'écharpe accroche une vis, un instant. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah pose l'écharpe près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. L'écharpe accroche une vis, un instant. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9247,7 +9247,7 @@
 narrateur|L'écharpe accroche une vis, un instant.
 narrateur|Un peu de poussière lève, puis retombe.
 narrateur|Sarah se cogne à son épaule, surprise.
-maman|Il a de l'élan, comme un petit vent.
+maman|Ses pieds veulent le haut, avant toi.
 papa|Toi tu as les jambes plus longues.
 enfant-f|On peut jouer avec lui ?
 papa|Vous trouvez, tous les deux ?</t>
@@ -9478,17 +9478,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose l'écharpe, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer.</t>
+          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose l'écharpe, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer. [pause]</t>
+          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9629,7 +9629,7 @@
 narrateur|Aniss va plus vite, Sarah plus loin.
 enfant-f|On arrive en haut, tous les deux.
 enfant-m|J'ai attendu ta jambe, un peu.
-papa|Vous avez joué avec l'élan.
+papa|Vos ombres ont monté ensemble.
 maman|Le marchepied vous a laissés passer.</t>
         </is>
       </c>
@@ -9850,17 +9850,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient l'écharpe, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois.</t>
+          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient l'écharpe, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois. [pause]</t>
+          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10002,7 +10002,7 @@
 enfant-m|C'est à toi, Sarah.
 enfant-f|Merci, j'y vais.
 papa|Chacun son tour, sur la marche.
-maman|L'élan a attendu le bois.</t>
+maman|Ses genoux ont reposé sur le bois.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr">
@@ -10221,17 +10221,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, dans sa paume. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu.</t>
+          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, dans sa paume. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman, tu tiens l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt; ? Je la donne, un coup chacun. Maman tient l'écharpe, dans sa paume. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman, tu tiens l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt; ? Je la donne, un coup chacun. Maman tient l'écharpe, dans sa paume. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt; ? Je la donne, un coup chacun. Maman tient l'écharpe, dans sa paume. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu. [pause]</t>
+          <t>Maman, tu tiens l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt; ? Je la donne, un coup chacun. Maman tient l'écharpe, dans sa paume. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10372,7 +10372,7 @@
 narrateur|Sarah la reçoit, monte plus loin.
 enfant-m|On demande, et ça va !
 enfant-f|Le haut est à nous.
-papa|Vous avez demandé, sans tirer.
+papa|Ma main tenait, vous montiez.
 maman|Ma main a juste attendu.</t>
         </is>
       </c>
@@ -10405,17 +10405,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. L'écharpe à pois marque le bois, un pois à la fois. Regarde-le, Aniss, il brille. Je le vois, d'ici. Une voix en haut, une voix en bas, puis plus.</t>
+          <t>Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. L'écharpe à pois marque le bois, un pois à la fois. Regarde-le, Aniss, il brille. Je le vois, d'ici. Une voix en haut, une voix en bas, puis plus.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. L'écharpe à pois marque le bois, un pois à la fois. Regarde-le, Aniss, il brille. Je le vois, d'ici. Une voix en haut, une voix en bas, puis plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. L'écharpe à pois marque le bois, un pois à la fois. Regarde-le, Aniss, il brille. Je le vois, d'ici. Une voix en haut, une voix en bas, puis plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. L'écharpe à pois marque le bois, un pois à la fois. Regarde-le, Aniss, il brille. Je le vois, d'ici. Une voix en haut, une voix en bas, puis plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. L'écharpe à pois marque le bois, un pois à la fois. Regarde-le, Aniss, il brille. Je le vois, d'ici. Une voix en haut, une voix en bas, puis plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10557,7 +10557,7 @@
 enfant-f|Maman a tendu l'écharpe.
 enfant-m|On s'est parlé à travers.
 papa|Le marchepied vous a laissé la place.
-maman|Le secret tient, tout chaud.
+maman|Le secret tient, chaud dans les mains.
 narrateur|L'écharpe à pois marque le bois, un pois à la fois.
 enfant-f|Regarde-le, Aniss, il brille.
 enfant-m|Je le vois, d'ici.
@@ -10593,17 +10593,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Sarah noue l'écharpe près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. L'écharpe claque contre le cou du cheval. L'écharpe attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Sarah noue l'écharpe près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. L'écharpe claque contre le cou du cheval. L'écharpe attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah noue l'écharpe près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. L'écharpe claque contre le cou du cheval. L'écharpe attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah noue l'écharpe près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. L'écharpe claque contre le cou du cheval. L'écharpe attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah noue l'écharpe près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. L'écharpe claque contre le cou du cheval. L'écharpe attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah noue l'écharpe près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. L'écharpe claque contre le cou du cheval. L'écharpe attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10745,11 +10745,11 @@
 enfant-f|Ici, ça brille, Aniss.
 enfant-f|Tu t'assois, et on tourne.
 enfant-m|Je galope, trop fort !
-narrateur|Le cheval doré penche, un tout petit peu.
+narrateur|Le cheval doré penche, un petit peu.
 narrateur|L'écharpe claque contre le cou du cheval.
 narrateur|L'écharpe attend au bord, un peu seule.
 narrateur|Sarah serre la selle, les dents serrées.
-maman|Son élan remplit tout le tour.
+maman|Ses genoux tapent la selle, trop fort.
 papa|Toi tu vas plus loin, lui plus vite.
 enfant-m|On tourne comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
@@ -11164,17 +11164,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La crinière sent le vernis, tout près. Le tour est à vous, maintenant. L'écharpe à pois pèse au cou, un peu lourde. Sarah la pose contre le bois peint. Un rai d'or traverse un pois, sur le cou.</t>
+          <t>Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La crinière sent le vernis, sous le nez. Le tour est à vous, maintenant. L'écharpe à pois pèse au cou, un peu lourde. Sarah la pose contre le bois peint. Un rai d'or traverse un pois, sur le cou.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis level="moderate"&gt;crinière&lt;/emphasis&gt; sent le vernis, tout près. Le tour est à vous, maintenant. L'écharpe à pois pèse au cou, un peu lourde. Sarah la pose contre le bois peint. Un rai d'or traverse un pois, sur le cou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis level="moderate"&gt;crinière&lt;/emphasis&gt; sent le vernis, sous le nez. Le tour est à vous, maintenant. L'écharpe à pois pèse au cou, un peu lourde. Sarah la pose contre le bois peint. Un rai d'or traverse un pois, sur le cou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis&gt;crinière&lt;/emphasis&gt; sent le vernis, tout près. Le tour est à vous, maintenant. L'écharpe à pois pèse au cou, un peu lourde. Sarah la pose contre le bois peint. Un rai d'or traverse un pois, sur le cou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis&gt;crinière&lt;/emphasis&gt; sent le vernis, sous le nez. Le tour est à vous, maintenant. L'écharpe à pois pèse au cou, un peu lourde. Sarah la pose contre le bois peint. Un rai d'or traverse un pois, sur le cou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11315,7 +11315,7 @@
           <t>narrateur|Les talons d'Aniss sont chauds, sur le bois.
 enfant-f|Tu as chanté pour moi.
 enfant-m|Tu tenais mon épaule.
-maman|La crinière sent le vernis, tout près.
+maman|La crinière sent le vernis, sous le nez.
 papa|Le tour est à vous, maintenant.
 narrateur|L'écharpe à pois pèse au cou, un peu lourde.
 narrateur|Sarah la pose contre le bois peint.
@@ -11351,17 +11351,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. L'écharpe à pois reste muette, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois.</t>
+          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. L'écharpe à pois reste muette, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'arrêt. Quand il s'arrête, on galope un peu. L'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt; à pois reste muette, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'arrêt. Quand il s'arrête, on galope un peu. L'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt; à pois reste muette, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. L'&lt;emphasis&gt;écharpe&lt;/emphasis&gt; à pois reste muette, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois. [pause]</t>
+          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. L'&lt;emphasis&gt;écharpe&lt;/emphasis&gt; à pois reste muette, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11498,12 +11498,12 @@
           <t>enfant-f|On attend l'arrêt.
 enfant-m|Quand il s'arrête, on galope un peu.
 narrateur|L'écharpe à pois reste muette, au creux.
-narrateur|Le cheval doré ralentit, tout seul.
+narrateur|Le cheval doré ralentit, sans nous.
 narrateur|Aniss souffle, puis il ouvre les mains.
 enfant-m|C'est à nous, maintenant.
 enfant-f|Un tour, sans galoper.
 papa|Vous avez attendu la musique.
-maman|L'élan a écouté le bois.</t>
+maman|Ses mains ont attendu le bois.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr">
@@ -11723,17 +11723,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près de l'écharpe. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu.</t>
+          <t>Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près de l'écharpe. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près de l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près de l'&lt;emphasis level="moderate"&gt;écharpe&lt;/emphasis&gt;. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près de l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu. [pause]</t>
+          <t>Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près de l'&lt;emphasis&gt;écharpe&lt;/emphasis&gt;. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11868,13 +11868,13 @@
       <c r="AW58" t="inlineStr">
         <is>
           <t>enfant-f|Papa, tu tiens la barre ?
-papa|Je la tiens, tout ferme.
+papa|Je la tiens, bien ferme.
 narrateur|Papa tient la barre, près de l'écharpe.
-narrateur|Aniss pose les deux mains, tout près.
+narrateur|Aniss pose les deux mains, contre la barre.
 narrateur|Sarah pose les siennes, plus loin.
 enfant-m|On demande, et ça tient !
 enfant-f|La crinière est à nous.
-maman|Vous avez demandé, sans galoper.
+maman|La barre tient, le cheval aussi.
 papa|Ma barre a juste attendu.</t>
         </is>
       </c>
@@ -13603,17 +13603,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, la clochette muette. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. La clochette ne bouge plus. Maintenant, c'est à nous.</t>
+          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, la clochette muette. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. La clochette ne bouge plus. Maintenant, c'est à nous.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; muette. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. La clochette ne bouge plus. Maintenant, c'est à nous.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; muette. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. La clochette ne bouge plus. Maintenant, c'est à nous.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, la &lt;emphasis&gt;clochette&lt;/emphasis&gt; muette. La file repose, toute ronde, toute sage. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. La clochette ne bouge plus. Maintenant, c'est à nous. [pause]</t>
+          <t>On attend un peu, Aniss. J'attends, je souffle. Aniss s'assoit près du kiosque, la &lt;emphasis&gt;clochette&lt;/emphasis&gt; muette. La file repose, ronde comme le kiosque. Sarah replace le pas, sans tirer. Tes pieds ont su s'asseoir. Le tour a eu la place. La clochette ne bouge plus. Maintenant, c'est à nous. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13750,7 +13750,7 @@
           <t>enfant-f|On attend un peu, Aniss.
 enfant-m|J'attends, je souffle.
 narrateur|Aniss s'assoit près du kiosque, la clochette muette.
-narrateur|La file repose, toute ronde, toute sage.
+narrateur|La file repose, ronde comme le kiosque.
 narrateur|Sarah replace le pas, sans tirer.
 papa|Tes pieds ont su s'asseoir.
 maman|Le tour a eu la place.
@@ -13787,17 +13787,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. La clochette reste dans la paume de Sarah. Je reste un peu. Un tintement mince s'endort près du kiosque.</t>
+          <t>Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. La clochette reste dans la paume de Sarah. Je reste un peu. Un tintement mince s'endort près du kiosque.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. La clochette reste dans la paume de Sarah. Je reste un peu. Un tintement mince s'endort près du kiosque.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. La clochette reste dans la paume de Sarah. Je reste un peu. Un tintement mince s'endort près du kiosque.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bord de la file, deux têtes se calment. Aniss, tu as su t'asseoir. Oui, tout près de tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. La clochette reste dans la paume de Sarah. Je reste un peu. Un tintement mince s'endort près du kiosque.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bord de la file, deux têtes se posent. Aniss, tu as su t'asseoir. Oui, contre tes mains. Toi debout, lui assis, ça tenait. Vos voix sont devenues toutes petites. La clochette reste dans la paume de Sarah. Je reste un peu. Un tintement mince s'endort près du kiosque.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13935,9 +13935,9 @@
       </c>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|Au bord de la file, deux têtes se calment.
+          <t>narrateur|Au bord de la file, deux têtes se posent.
 enfant-f|Aniss, tu as su t'asseoir.
-enfant-m|Oui, tout près de tes mains.
+enfant-m|Oui, contre tes mains.
 papa|Toi debout, lui assis, ça tenait.
 maman|Vos voix sont devenues toutes petites.
 narrateur|La clochette reste dans la paume de Sarah.
@@ -13974,17 +13974,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, loin de la clochette. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. La clochette reste près d'eux. La file est prête.</t>
+          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, loin de la clochette. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. La clochette reste près d'eux. La file est prête.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, loin de la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. La clochette reste près d'eux. La file est prête.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, loin de la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. La clochette reste près d'eux. La file est prête.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, loin de la &lt;emphasis&gt;clochette&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Vous avez demandé, et ça tient. La clochette reste près d'eux. La file est prête. [pause]</t>
+          <t>Papa, tu le tiens ? Je le tiens, Sarah. Papa tient le ticket, loin de la &lt;emphasis&gt;clochette&lt;/emphasis&gt;. Les mains d'Aniss sont libres, maintenant. Sarah avance d'un pas, pile au milieu. Je t'aide, sans le ticket. Papa a le papier, vos mains sont libres. La clochette reste près d'eux. La file est prête. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14124,7 +14124,7 @@
 narrateur|Les mains d'Aniss sont libres, maintenant.
 narrateur|Sarah avance d'un pas, pile au milieu.
 enfant-m|Je t'aide, sans le ticket.
-maman|Vous avez demandé, et ça tient.
+maman|Papa a le papier, vos mains sont libres.
 narrateur|La clochette reste près d'eux.
 enfant-f|La file est prête.</t>
         </is>
@@ -14345,17 +14345,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose la clochette près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. La clochette tape le fer, toc. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Sarah pose la clochette près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. La clochette tape le fer, toc. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. La clochette tape le fer, toc. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. La clochette tape le fer, toc. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah pose la &lt;emphasis&gt;clochette&lt;/emphasis&gt; près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. La clochette tape le fer, toc. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Il a de l'élan, comme un petit vent. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah pose la &lt;emphasis&gt;clochette&lt;/emphasis&gt; près du marchepied. Le marchepied est à nous, Aniss. Moi je monte, tu me suis. Je monte le premier, trop vite ! Ses pieds quittent le sol, puis reviennent. La clochette tape le fer, toc. Un peu de poussière lève, puis retombe. Sarah se cogne à son épaule, surprise. Ses pieds veulent le haut, avant toi. Toi tu as les jambes plus longues. On peut jouer avec lui ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14501,7 +14501,7 @@
 narrateur|La clochette tape le fer, toc.
 narrateur|Un peu de poussière lève, puis retombe.
 narrateur|Sarah se cogne à son épaule, surprise.
-maman|Il a de l'élan, comme un petit vent.
+maman|Ses pieds veulent le haut, avant toi.
 papa|Toi tu as les jambes plus longues.
 enfant-f|On peut jouer avec lui ?
 papa|Vous trouvez, tous les deux ?</t>
@@ -14732,17 +14732,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose la clochette, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer.</t>
+          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose la clochette, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose la &lt;emphasis&gt;clochette&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vous avez joué avec l'élan. Le marchepied vous a laissés passer. [pause]</t>
+          <t>On monte ensemble, Aniss. Toi derrière, moi devant ! Sarah pose la &lt;emphasis&gt;clochette&lt;/emphasis&gt;, sans bruit, sur le bois. Deux ombres montent sur la même marche. Aniss va plus vite, Sarah plus loin. On arrive en haut, tous les deux. J'ai attendu ta jambe, un peu. Vos ombres ont monté ensemble. Le marchepied vous a laissés passer. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14883,7 +14883,7 @@
 narrateur|Aniss va plus vite, Sarah plus loin.
 enfant-f|On arrive en haut, tous les deux.
 enfant-m|J'ai attendu ta jambe, un peu.
-papa|Vous avez joué avec l'élan.
+papa|Vos ombres ont monté ensemble.
 maman|Le marchepied vous a laissés passer.</t>
         </is>
       </c>
@@ -15104,17 +15104,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient la clochette, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois.</t>
+          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient la clochette, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient la &lt;emphasis&gt;clochette&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. L'élan a attendu le bois. [pause]</t>
+          <t>On s'assoit un peu. Moi je m'assois, puis c'est toi. Sarah tient la &lt;emphasis&gt;clochette&lt;/emphasis&gt;, sur la marche. Aniss pose les genoux sur le bois. Il souffle, puis il se lève. C'est à toi, Sarah. Merci, j'y vais. Chacun son tour, sur la marche. Ses genoux ont reposé sur le bois. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15256,7 +15256,7 @@
 enfant-m|C'est à toi, Sarah.
 enfant-f|Merci, j'y vais.
 papa|Chacun son tour, sur la marche.
-maman|L'élan a attendu le bois.</t>
+maman|Ses genoux ont reposé sur le bois.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
@@ -15475,17 +15475,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près de la clochette. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu.</t>
+          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près de la clochette. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près de la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près de la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près de la &lt;emphasis&gt;clochette&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Vous avez demandé, sans tirer. Ma main a juste attendu. [pause]</t>
+          <t>Maman, tu tiens l'écharpe ? Je la donne, un coup chacun. Maman tient l'écharpe, près de la &lt;emphasis&gt;clochette&lt;/emphasis&gt;. Aniss la reçoit, monte un pas. Sarah la reçoit, monte plus loin. On demande, et ça va ! Le haut est à nous. Ma main tenait, vous montiez. Ma main a juste attendu. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15626,7 +15626,7 @@
 narrateur|Sarah la reçoit, monte plus loin.
 enfant-m|On demande, et ça va !
 enfant-f|Le haut est à nous.
-papa|Vous avez demandé, sans tirer.
+papa|Ma main tenait, vous montiez.
 maman|Ma main a juste attendu.</t>
         </is>
       </c>
@@ -15659,17 +15659,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. La clochette marque le bois d'un toc heureux. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le toc heureux s'endort sur la marche.</t>
+          <t>Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. La clochette marque le bois d'un toc heureux. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le toc heureux s'endort sur la marche.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. La clochette marque le bois d'un toc heureux. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le toc heureux s'endort sur la marche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. La clochette marque le bois d'un toc heureux. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le toc heureux s'endort sur la marche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, tout chaud. La clochette marque le bois d'un toc heureux. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le toc heureux s'endort sur la marche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une voix en haut, une voix en bas, puis plus. Maman a tendu l'écharpe. On s'est parlé à travers. Le marchepied vous a laissé la place. Le secret tient, chaud dans les mains. La clochette marque le bois d'un toc heureux. Regarde-le, Aniss, il brille. Je le vois, d'ici. Le toc heureux s'endort sur la marche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15811,7 +15811,7 @@
 enfant-f|Maman a tendu l'écharpe.
 enfant-m|On s'est parlé à travers.
 papa|Le marchepied vous a laissé la place.
-maman|Le secret tient, tout chaud.
+maman|Le secret tient, chaud dans les mains.
 narrateur|La clochette marque le bois d'un toc heureux.
 enfant-f|Regarde-le, Aniss, il brille.
 enfant-m|Je le vois, d'ici.
@@ -15847,17 +15847,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose la clochette près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. La clochette tinte trop près de l'oreille. La clochette attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Sarah pose la clochette près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. La clochette tinte trop près de l'oreille. La clochette attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. La clochette tinte trop près de l'oreille. La clochette attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah pose la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. La clochette tinte trop près de l'oreille. La clochette attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah pose la &lt;emphasis&gt;clochette&lt;/emphasis&gt; près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un tout petit peu. La clochette tinte trop près de l'oreille. La clochette attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Son élan remplit tout le tour. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah pose la &lt;emphasis&gt;clochette&lt;/emphasis&gt; près de la crinière. Ici, ça brille, Aniss. Tu t'assois, et on tourne. Je galope, trop fort ! Le cheval doré penche, un petit peu. La clochette tinte trop près de l'oreille. La clochette attend au bord, un peu seule. Sarah serre la selle, les dents serrées. Ses genoux tapent la selle, trop fort. Toi tu vas plus loin, lui plus vite. On tourne comment, alors ? Vous trouvez, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15999,11 +15999,11 @@
 enfant-f|Ici, ça brille, Aniss.
 enfant-f|Tu t'assois, et on tourne.
 enfant-m|Je galope, trop fort !
-narrateur|Le cheval doré penche, un tout petit peu.
+narrateur|Le cheval doré penche, un petit peu.
 narrateur|La clochette tinte trop près de l'oreille.
 narrateur|La clochette attend au bord, un peu seule.
 narrateur|Sarah serre la selle, les dents serrées.
-maman|Son élan remplit tout le tour.
+maman|Ses genoux tapent la selle, trop fort.
 papa|Toi tu vas plus loin, lui plus vite.
 enfant-m|On tourne comment, alors ?
 papa|Vous trouvez, tous les deux ?</t>
@@ -16418,17 +16418,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La crinière sent le vernis, tout près. Le tour est à vous, maintenant. La clochette pèse au poignet, un peu lourde. Sarah la pose contre le bois peint. La valse redevient petite, près du poignet.</t>
+          <t>Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La crinière sent le vernis, sous le nez. Le tour est à vous, maintenant. La clochette pèse au poignet, un peu lourde. Sarah la pose contre le bois peint. La valse redevient petite, près du poignet.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis level="moderate"&gt;crinière&lt;/emphasis&gt; sent le vernis, tout près. Le tour est à vous, maintenant. La clochette pèse au poignet, un peu lourde. Sarah la pose contre le bois peint. La valse redevient petite, près du poignet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis level="moderate"&gt;crinière&lt;/emphasis&gt; sent le vernis, sous le nez. Le tour est à vous, maintenant. La clochette pèse au poignet, un peu lourde. Sarah la pose contre le bois peint. La valse redevient petite, près du poignet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis&gt;crinière&lt;/emphasis&gt; sent le vernis, tout près. Le tour est à vous, maintenant. La clochette pèse au poignet, un peu lourde. Sarah la pose contre le bois peint. La valse redevient petite, près du poignet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons d'Aniss sont chauds, sur le bois. Tu as chanté pour moi. Tu tenais mon épaule. La &lt;emphasis&gt;crinière&lt;/emphasis&gt; sent le vernis, sous le nez. Le tour est à vous, maintenant. La clochette pèse au poignet, un peu lourde. Sarah la pose contre le bois peint. La valse redevient petite, près du poignet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16569,7 +16569,7 @@
           <t>narrateur|Les talons d'Aniss sont chauds, sur le bois.
 enfant-f|Tu as chanté pour moi.
 enfant-m|Tu tenais mon épaule.
-maman|La crinière sent le vernis, tout près.
+maman|La crinière sent le vernis, sous le nez.
 papa|Le tour est à vous, maintenant.
 narrateur|La clochette pèse au poignet, un peu lourde.
 narrateur|Sarah la pose contre le bois peint.
@@ -16605,17 +16605,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. La clochette reste muette, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois.</t>
+          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. La clochette reste muette, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'arrêt. Quand il s'arrête, on galope un peu. La &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; reste muette, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'arrêt. Quand il s'arrête, on galope un peu. La &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt; reste muette, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. La &lt;emphasis&gt;clochette&lt;/emphasis&gt; reste muette, au creux. Le cheval doré ralentit, tout seul. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. L'élan a écouté le bois. [pause]</t>
+          <t>On attend l'arrêt. Quand il s'arrête, on galope un peu. La &lt;emphasis&gt;clochette&lt;/emphasis&gt; reste muette, au creux. Le cheval doré ralentit, sans nous. Aniss souffle, puis il ouvre les mains. C'est à nous, maintenant. Un tour, sans galoper. Vous avez attendu la musique. Ses mains ont attendu le bois. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16752,12 +16752,12 @@
           <t>enfant-f|On attend l'arrêt.
 enfant-m|Quand il s'arrête, on galope un peu.
 narrateur|La clochette reste muette, au creux.
-narrateur|Le cheval doré ralentit, tout seul.
+narrateur|Le cheval doré ralentit, sans nous.
 narrateur|Aniss souffle, puis il ouvre les mains.
 enfant-m|C'est à nous, maintenant.
 enfant-f|Un tour, sans galoper.
 papa|Vous avez attendu la musique.
-maman|L'élan a écouté le bois.</t>
+maman|Ses mains ont attendu le bois.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr">
@@ -16977,17 +16977,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près de la clochette. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu.</t>
+          <t>Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près de la clochette. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près de la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près de la &lt;emphasis level="moderate"&gt;clochette&lt;/emphasis&gt;. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu tiens la barre ? Je la tiens, tout ferme. Papa tient la barre, près de la &lt;emphasis&gt;clochette&lt;/emphasis&gt;. Aniss pose les deux mains, tout près. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. Vous avez demandé, sans galoper. Ma barre a juste attendu. [pause]</t>
+          <t>Papa, tu tiens la barre ? Je la tiens, bien ferme. Papa tient la barre, près de la &lt;emphasis&gt;clochette&lt;/emphasis&gt;. Aniss pose les deux mains, contre la barre. Sarah pose les siennes, plus loin. On demande, et ça tient ! La crinière est à nous. La barre tient, le cheval aussi. Ma barre a juste attendu. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17122,13 +17122,13 @@
       <c r="AW86" t="inlineStr">
         <is>
           <t>enfant-f|Papa, tu tiens la barre ?
-papa|Je la tiens, tout ferme.
+papa|Je la tiens, bien ferme.
 narrateur|Papa tient la barre, près de la clochette.
-narrateur|Aniss pose les deux mains, tout près.
+narrateur|Aniss pose les deux mains, contre la barre.
 narrateur|Sarah pose les siennes, plus loin.
 enfant-m|On demande, et ça tient !
 enfant-f|La crinière est à nous.
-maman|Vous avez demandé, sans galoper.
+maman|La barre tient, le cheval aussi.
 papa|Ma barre a juste attendu.</t>
         </is>
       </c>
@@ -17343,7 +17343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17456,6 +17456,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>